<commit_message>
datos de densidades: control de variables
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\physics-graphs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90E10F97-7B55-4F72-9549-BD78613B5B8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDEE46C8-74B1-4D3C-A897-4A55072AC85C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{92CE9620-F6EB-4642-991A-68F408009301}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="3" xr2:uid="{92CE9620-F6EB-4642-991A-68F408009301}"/>
   </bookViews>
   <sheets>
     <sheet name="pendulo" sheetId="1" r:id="rId1"/>
     <sheet name="resorte" sheetId="2" r:id="rId2"/>
+    <sheet name="analisis" sheetId="3" r:id="rId3"/>
+    <sheet name="analisis2" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>L</t>
   </si>
@@ -49,12 +51,42 @@
   </si>
   <si>
     <t>d</t>
+  </si>
+  <si>
+    <t>p0.7</t>
+  </si>
+  <si>
+    <t>p1.5</t>
+  </si>
+  <si>
+    <t>p2.1</t>
+  </si>
+  <si>
+    <t>p3.2</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>q1</t>
+  </si>
+  <si>
+    <t>q1.5</t>
+  </si>
+  <si>
+    <t>q2.0</t>
+  </si>
+  <si>
+    <t>q4.0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -84,8 +116,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -536,4 +570,194 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB0FB347-92AA-4E4B-BC3A-5C72D03CB11D}">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1">
+        <v>25</v>
+      </c>
+      <c r="C2">
+        <v>16.5</v>
+      </c>
+      <c r="D2" s="1">
+        <v>14</v>
+      </c>
+      <c r="E2" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1.5</v>
+      </c>
+      <c r="B3">
+        <v>52.5</v>
+      </c>
+      <c r="C3">
+        <v>35.799999999999997</v>
+      </c>
+      <c r="D3">
+        <v>30.5</v>
+      </c>
+      <c r="E3">
+        <v>24.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1">
+        <v>95</v>
+      </c>
+      <c r="C4">
+        <v>65.2</v>
+      </c>
+      <c r="D4">
+        <v>55.1</v>
+      </c>
+      <c r="E4" s="2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1">
+        <v>381</v>
+      </c>
+      <c r="C5">
+        <v>261.10000000000002</v>
+      </c>
+      <c r="D5">
+        <v>231.1</v>
+      </c>
+      <c r="E5" s="1">
+        <v>179</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E740D31A-D35C-4EB5-98AA-BA2FCBF89916}">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0.7</v>
+      </c>
+      <c r="B2" s="1">
+        <v>25</v>
+      </c>
+      <c r="C2">
+        <v>52.5</v>
+      </c>
+      <c r="D2" s="1">
+        <v>95</v>
+      </c>
+      <c r="E2" s="1">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1.5</v>
+      </c>
+      <c r="B3">
+        <v>16.5</v>
+      </c>
+      <c r="C3">
+        <v>35.799999999999997</v>
+      </c>
+      <c r="D3">
+        <v>65.2</v>
+      </c>
+      <c r="E3">
+        <v>261.10000000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2.1</v>
+      </c>
+      <c r="B4" s="2">
+        <v>14</v>
+      </c>
+      <c r="C4">
+        <v>30.5</v>
+      </c>
+      <c r="D4">
+        <v>55.1</v>
+      </c>
+      <c r="E4">
+        <v>231.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3.2</v>
+      </c>
+      <c r="B5" s="2">
+        <v>11</v>
+      </c>
+      <c r="C5">
+        <v>24.8</v>
+      </c>
+      <c r="D5" s="2">
+        <v>45</v>
+      </c>
+      <c r="E5" s="2">
+        <v>179</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
todos los problemas graficados
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,15 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\physics-graphs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDEE46C8-74B1-4D3C-A897-4A55072AC85C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8A3E1F9-231F-4DE4-8E0F-A7B67F04B205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="3" xr2:uid="{92CE9620-F6EB-4642-991A-68F408009301}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="8" xr2:uid="{92CE9620-F6EB-4642-991A-68F408009301}"/>
   </bookViews>
   <sheets>
     <sheet name="pendulo" sheetId="1" r:id="rId1"/>
     <sheet name="resorte" sheetId="2" r:id="rId2"/>
     <sheet name="analisis" sheetId="3" r:id="rId3"/>
     <sheet name="analisis2" sheetId="4" r:id="rId4"/>
+    <sheet name="P31" sheetId="6" r:id="rId5"/>
+    <sheet name="P38" sheetId="7" r:id="rId6"/>
+    <sheet name="P44" sheetId="8" r:id="rId7"/>
+    <sheet name="P56" sheetId="5" r:id="rId8"/>
+    <sheet name="P57" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
   <si>
     <t>L</t>
   </si>
@@ -78,14 +83,33 @@
   </si>
   <si>
     <t>q4.0</t>
+  </si>
+  <si>
+    <t>Q</t>
+  </si>
+  <si>
+    <t>V</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>P</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.000E+00"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -116,10 +140,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -760,4 +785,310 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A0343885-C397-4520-8D5F-23D5BCB817C1}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>20</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{755D5067-9C1B-4878-A52D-4292CCFD53DC}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>9</v>
+      </c>
+      <c r="B5">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>10</v>
+      </c>
+      <c r="B6">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>13</v>
+      </c>
+      <c r="B7">
+        <v>531</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{217A10E9-2583-4B39-B9C5-AA127B6B4577}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0.5</v>
+      </c>
+      <c r="B2">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>0.75</v>
+      </c>
+      <c r="B3">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>1.25</v>
+      </c>
+      <c r="B4">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>1.5</v>
+      </c>
+      <c r="B5">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>1.75</v>
+      </c>
+      <c r="B6">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39273DD2-437F-4A78-B9CF-AA3B096D2CB6}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>74.099999999999994</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>40</v>
+      </c>
+      <c r="B3">
+        <v>30.1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>60</v>
+      </c>
+      <c r="B4">
+        <v>16.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>90</v>
+      </c>
+      <c r="B5">
+        <v>6.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>100</v>
+      </c>
+      <c r="B6" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>150</v>
+      </c>
+      <c r="B7">
+        <v>1.1000000000000001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ADC61C57-D69E-4F9D-B098-F5D5382D2371}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2" s="3">
+        <v>1177000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>10</v>
+      </c>
+      <c r="B3" s="3">
+        <v>1438000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>20</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1756000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>30</v>
+      </c>
+      <c r="B5" s="3">
+        <v>2144000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>50</v>
+      </c>
+      <c r="B6" s="3">
+        <v>3199000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>